<commit_message>
Initialted implementation of Login test
</commit_message>
<xml_diff>
--- a/data_files/login_data.xlsx
+++ b/data_files/login_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EXPLEO SMARTCLIFF\Phase - 9 Automation Testing Using Python\TutorialsNinja\DataFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SOURCE CODE\Python Automation\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69A1921-5C9E-413D-87F4-22CADD8636F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{528CCD00-14C6-4420-A61D-651FAE22D712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{1CB0E6C3-1D2C-4AF9-B615-C9DA0459DFE3}"/>
   </bookViews>
@@ -38,10 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
-  <si>
-    <t>username</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>password</t>
   </si>
@@ -49,26 +46,56 @@
     <t>admin</t>
   </si>
   <si>
-    <t>hlhl@gmail.com</t>
-  </si>
-  <si>
     <t>error message</t>
   </si>
   <si>
-    <t>admin123</t>
-  </si>
-  <si>
-    <t>hlhls@gmail.com</t>
-  </si>
-  <si>
-    <t>Warning: No match for E-Mail Address and/or Password.</t>
+    <t>role</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Doctor</t>
+  </si>
+  <si>
+    <t>Pharmacist</t>
+  </si>
+  <si>
+    <t>Pathologist</t>
+  </si>
+  <si>
+    <t>Radiologist</t>
+  </si>
+  <si>
+    <t>Accountant</t>
+  </si>
+  <si>
+    <t>Receptionist</t>
+  </si>
+  <si>
+    <t>Nurse</t>
+  </si>
+  <si>
+    <t>Super Admin</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>superadmin@gmail.com</t>
+  </si>
+  <si>
+    <t>super.admin@gmail.com</t>
+  </si>
+  <si>
+    <t>Invalid Username or Password</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -85,7 +112,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -112,10 +151,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -431,40 +474,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59122902-2086-4E9C-9EBC-01EE140966BE}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{E3DA01C9-6AA5-4F33-9773-F6FF48305560}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -474,42 +540,42 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>